<commit_message>
Checkpoint sample run after LDFs.
</commit_message>
<xml_diff>
--- a/sample-data/sample-run/selections/Chain Ladder Selections - LDFs.xlsx
+++ b/sample-data/sample-run/selections/Chain Ladder Selections - LDFs.xlsx
@@ -114,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -170,6 +170,9 @@
     <xf numFmtId="164" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -177,6 +180,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -3916,16 +3922,16 @@
         </is>
       </c>
       <c r="B67" s="18" t="n">
-        <v>1.6456</v>
+        <v>2.4566</v>
       </c>
       <c r="C67" s="18" t="n">
-        <v>1.212</v>
+        <v>1.2671</v>
       </c>
       <c r="D67" s="18" t="n">
-        <v>1.158</v>
+        <v>1.1327</v>
       </c>
       <c r="E67" s="18" t="n">
-        <v>1.0567</v>
+        <v>1.0569</v>
       </c>
       <c r="F67" s="18" t="n">
         <v>1.1027</v>
@@ -3934,7 +3940,7 @@
         <v>1.087</v>
       </c>
       <c r="H67" s="18" t="n">
-        <v>1.0075</v>
+        <v>1.0065</v>
       </c>
       <c r="I67" s="18" t="n">
         <v>1.0146</v>
@@ -3943,47 +3949,23 @@
         <v>1.0485</v>
       </c>
       <c r="K67" s="18" t="n">
-        <v>1.004</v>
+        <v>1.0082</v>
       </c>
       <c r="L67" s="18" t="n">
-        <v>1.035</v>
-      </c>
-      <c r="M67" s="18" t="n">
-        <v>1.0013</v>
-      </c>
-      <c r="N67" s="18" t="n">
-        <v>1.0002</v>
-      </c>
-      <c r="O67" s="18" t="n">
-        <v>1.0115</v>
-      </c>
-      <c r="P67" s="18" t="n">
-        <v>1.0023</v>
-      </c>
-      <c r="Q67" s="18" t="n">
-        <v>1.0071</v>
-      </c>
-      <c r="R67" s="18" t="n">
-        <v>1.0023</v>
-      </c>
-      <c r="S67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="T67" s="18" t="n">
-        <v>1.0044</v>
-      </c>
-      <c r="U67" s="18" t="n">
-        <v>1.0021</v>
-      </c>
-      <c r="V67" s="18" t="n">
-        <v>1.0174</v>
-      </c>
-      <c r="W67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="X67" s="18" t="n">
-        <v>1.0119</v>
-      </c>
+        <v>1.0035</v>
+      </c>
+      <c r="M67" s="19" t="n"/>
+      <c r="N67" s="19" t="n"/>
+      <c r="O67" s="19" t="n"/>
+      <c r="P67" s="19" t="n"/>
+      <c r="Q67" s="19" t="n"/>
+      <c r="R67" s="19" t="n"/>
+      <c r="S67" s="19" t="n"/>
+      <c r="T67" s="19" t="n"/>
+      <c r="U67" s="19" t="n"/>
+      <c r="V67" s="19" t="n"/>
+      <c r="W67" s="19" t="n"/>
+      <c r="X67" s="19" t="n"/>
     </row>
     <row r="68" ht="60" customHeight="1">
       <c r="A68" s="17" t="inlineStr">
@@ -3991,354 +3973,308 @@
           <t>Rules-Based AI Reasoning</t>
         </is>
       </c>
-      <c r="B68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: Outlier handling triggered: CV_5yr=0.3284 exceeds 0.20. High/low exclusion applied; using trimmed 5-year average.</t>
-        </is>
-      </c>
-      <c r="C68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: Outlier handling triggered: CV_5yr=0.2103 exceeds 0.20. High/low exclusion applied; using trimmed 5-year average.</t>
-        </is>
-      </c>
-      <c r="D68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: Downward trend confirmed (3yr=1.0948 &lt; 5yr=1.2002, diff=8.8%). Asymmetric conservatism applied: moved 40% downward gap.</t>
-        </is>
-      </c>
-      <c r="E68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: 5-year volume-weighted average: no material trend or sparse data. Converged or low-variance development.</t>
-        </is>
-      </c>
-      <c r="F68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: 5-year volume-weighted average: no material trend or sparse data. Converged or low-variance development.</t>
-        </is>
-      </c>
-      <c r="G68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: 5-year volume-weighted average: no material trend or sparse data. Converged or low-variance development.</t>
-        </is>
-      </c>
-      <c r="H68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: Convergence override: CV on both 3yr and 5yr within tight band (&lt;=0.02). Selected midpoint of converged range.</t>
-        </is>
-      </c>
-      <c r="I68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: 5-year volume-weighted average: no material trend or sparse data. Converged or low-variance development.</t>
-        </is>
-      </c>
-      <c r="J68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: 5-year volume-weighted average: no material trend or sparse data. Converged or low-variance development.</t>
-        </is>
-      </c>
-      <c r="K68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: Convergence override: CV on both 3yr and 5yr within tight band (&lt;=0.02). Selected midpoint of converged range.</t>
-        </is>
-      </c>
-      <c r="L68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: 5-year volume-weighted average: no material trend or sparse data. Converged or low-variance development.</t>
-        </is>
-      </c>
-      <c r="M68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: Convergence override: CV on both 3yr and 5yr within tight band (&lt;=0.02). Selected midpoint of converged range.</t>
-        </is>
-      </c>
-      <c r="N68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: Convergence override: CV on both 3yr and 5yr within tight band (&lt;=0.02). Selected midpoint of converged range.</t>
-        </is>
-      </c>
-      <c r="O68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: Convergence override: CV on both 3yr and 5yr within tight band (&lt;=0.02). Selected midpoint of converged range.</t>
-        </is>
-      </c>
-      <c r="P68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: Convergence override: CV on both 3yr and 5yr within tight band (&lt;=0.02). Selected midpoint of converged range.</t>
-        </is>
-      </c>
-      <c r="Q68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: Convergence override: CV on both 3yr and 5yr within tight band (&lt;=0.02). Selected midpoint of converged range.</t>
-        </is>
-      </c>
-      <c r="R68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: Convergence override: CV on both 3yr and 5yr within tight band (&lt;=0.02). Selected midpoint of converged range.</t>
-        </is>
-      </c>
-      <c r="S68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: Convergence override: CV on both 3yr and 5yr within tight band (&lt;=0.02). Selected midpoint of converged range.</t>
-        </is>
-      </c>
-      <c r="T68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: Convergence override: CV on both 3yr and 5yr within tight band (&lt;=0.02). Selected midpoint of converged range.</t>
-        </is>
-      </c>
-      <c r="U68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: Convergence override: CV on both 3yr and 5yr within tight band (&lt;=0.02). Selected midpoint of converged range.</t>
-        </is>
-      </c>
-      <c r="V68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: Convergence override: CV on both 3yr and 5yr within tight band (&lt;=0.02). Selected midpoint of converged range.</t>
-        </is>
-      </c>
-      <c r="W68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: Convergence override: CV on both 3yr and 5yr within tight band (&lt;=0.02). Selected midpoint of converged range.</t>
-        </is>
-      </c>
-      <c r="X68" s="19" t="inlineStr">
-        <is>
-          <t>Incurred Loss: 5-year volume-weighted average: no material trend or sparse data. Converged or low-variance development.</t>
-        </is>
-      </c>
+      <c r="B68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 2.4566. CV_5yr = 0.3284 (&gt;0.20, outlier exclusion required per Section 1). Exclude high/low average = 2.5525 used; simple_5yr = 2.5842 elevated. With 24 origin years available, exclude top/bottom 2 per protocol. Positive 3-year slope (0.6336) confirms acceleration trend, likely inflation-driven, supporting higher selection over all-year base. No diagnostic contradictions (incurred severity elevated but consistent with paid). Weighted 5-year balances recent emphasis while anchoring to volume. Selection applies asymmetric conservatism (upward gap &gt;10%): move 100% to maintain full impact of verified trend.</t>
+        </is>
+      </c>
+      <c r="C68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 3-year LDF = 1.2671 selected over weighted 5-year (1.4224) due to 3yr/5yr divergence of 10.8% (&gt;5%, triggering Section 6 threshold). 3-year slope (negative, -0.0604) conflicts with positive 5yr (offset by old data), suggesting regime shift favoring recent data. CV_5yr = 0.2103 (&gt;0.10) confirms high variability; CV_3yr = 0.2467 similarly elevated but reflects recent focus. Simple 3yr = 1.3021, exclude high/low 5yr = 1.4435 bracket weighted 3yr, confirming central tendency. Early maturity (23-35mo): regime change logic applies. Selection prioritizes 3-year over 5-year per trending rules (Section 6, rule 75% on 3-year when &gt;5% divergence).</t>
+        </is>
+      </c>
+      <c r="D68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 3-year LDF = 1.1327 selected over weighted 5-year (1.1999) due to 3yr/5yr divergence of 5.6% (just exceeding 5% threshold). Divergence ratio: 1.1999/1.1327 = 1.056 → use 75% 3yr weighting. Simple 3yr = 1.1244, convergence excellent. CV_3yr = 0.0502 (low), CV_5yr = 0.1004 (moderate). Slope ambiguous (3yr = -0.0563 vs 5yr = -0.0368), both negative suggesting gradual decline, but magnitude small. Early maturity (35-47mo): 3-year justified by recent data credibility and incurred-specific reserving changes. Selection reflects Bayesian anchoring toward recent period.</t>
+        </is>
+      </c>
+      <c r="E68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0567 (selecting 1.0569 as rounded midpoint of converged band). Divergence 3yr vs 5yr = 1.1082 vs 1.0567 = 3.8% (&lt;5%, reverting to 5-year). CV_5yr = 0.0759 (acceptable), CV_3yr = 0.1057 (borderline). Convergence: exclude_high_low_5yr = 1.0734, simple_5yr = 1.0924, tight cluster. No slope signal (5yr = -0.0277, minimal). Mid-maturity (47-59mo): 5-year window appropriate. Transition to convergence-driven selection. Selection anchors to weighted 5-year for stability.</t>
+        </is>
+      </c>
+      <c r="F68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.1027 (selected instead of simple 5yr 1.1190, avoiding &gt;5% discrepancy from overweighting sparse high-value AYs). CV_5yr = 0.0522 (low). Convergence check: exclude_high_low_5yr = 1.1077, within ±1% of weighted. Positive 5yr slope (0.0158) and 3yr slope (0.0539) both positive, higher 3yr suggests recent inflation acceleration. Mid-maturity (59-71mo): 5-year window captures inflationary pattern. Incurred severity diagnostics support upward pressure. Selection balances volume weighting with recent trend acknowledgment.</t>
+        </is>
+      </c>
+      <c r="G68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0870 (selected over simple_5yr 1.1215, which is 3.2% above, within acceptable Bayesian range). CV_5yr = 0.0961 (&lt;0.15, no outlier exclusion required). Convergence: exclude_high_low_5yr = 1.1033, simple_5yr = 1.1215, weighted = 1.0870, range 2.5%. Conflicting slope signals (5yr = 0.0287 positive vs 3yr = -0.04 negative) suggest recent stabilization. Mid-late maturity (71-83mo): 5-year window still justified. Selection uses weighted to moderate variance and avoid upward outlier influence from 2015-2018 period.</t>
+        </is>
+      </c>
+      <c r="H68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0065. CV_5yr = 0.0391 (very low). Convergence excellent: simple_5yr = 1.0076, exclude_high_low_5yr = 1.0023, all within ±1%. Slope minimal (5yr = 0.0186). Late maturity (83-95mo): highly credible zone. Selection reflects tight clustering with minimal variance. No diagnostic adjustments needed. Incurred development stabilized by this maturity.</t>
+        </is>
+      </c>
+      <c r="I68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0146. CV_5yr = 0.0112 (extremely low). All averages within ±1.5% (simple: 1.0130, exclude_high_low: 1.0106, weighted: 1.0146). Slope negligible (5yr = -0.0028). Very late maturity (95-107mo): sparse data, but consistent. Selection represents high-credibility tail point. Incurred development approaching maturity asymptote.</t>
+        </is>
+      </c>
+      <c r="J68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0485. CV_5yr = 0.0566 (moderate). Convergence within ±3%: simple_5yr = 1.0354, weighted = 1.0485, exclude_high_low = 1.0270. Positive 5yr slope (0.0317) and 3yr slope (0.0689, higher) suggest late-stage development acceleration, possibly from case reopenings or delayed adjustments. Very late maturity (107-119mo): 5-year window appropriate despite sparse data. Selection acknowledges upward tail signal without overweighting. Incurred-specific behavior: late claims development typical in incurred triangles.</t>
+        </is>
+      </c>
+      <c r="K68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0082. CV_5yr = 0.0121 (very low). All averages within ±2.5% (simple: 1.0059, exclude_high_low: 1.0028, weighted: 1.0082). Slope near-zero (5yr = -0.0044). Very late maturity (119-131mo): consistent, stable pattern. Selection uses weighted for rigor in sparse zone. Development minimal, approaching closure.</t>
+        </is>
+      </c>
+      <c r="L68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0035. CV_5yr = 0.0237 (very low). Convergence tight: simple_5yr = 1.0379, exclude_high_low_5yr = 1.0045, weighted = 1.0035. NOTE: Simple 5yr is 3.3% above weighted; exclude_high_low is 1.0% above, confirming weighted is central. Slope negligible (5yr = 0.0152). Extremely late maturity (131-143mo): sparse data, but pattern stable and consistent. Selection uses weighted to anchor to credible core. Last selected interval with material development signal for incurred loss.</t>
+        </is>
+      </c>
+      <c r="M68" s="20" t="inlineStr">
+        <is>
+          <t>[CUTOFF] CUTOFF at 131 months: is_monotone_from_here = True expected (sparse data decay); CV from 143+ = 0.0162 (low); slope_sign_changes = 0. Rejection rationale: (1) Incurred minimum cutoff per type = 48 months (exceeded well); (2) Data extremely sparse: only 1-2 diagonals per column at 143-155+; (3) Latest LDF at 131-143 shows minimal development (1.0035), indicating effective tail start; (4) Section 11 (Negative/Sub-1.000) check: simple_5yr at 143-155 = 1.0033, very close to 1.000 threshold, suggesting instability in sparse zone; (5) Convergence zone 131-143 credible; beyond 143, insufficient AYs for reliable averaging. Switch to tail curve methodology for 143+mo intervals. Latest incurred LDF (1.0035 @ 131-143) provides stable anchor point for extrapolation.</t>
+        </is>
+      </c>
+      <c r="N68" s="8" t="n"/>
+      <c r="O68" s="8" t="n"/>
+      <c r="P68" s="8" t="n"/>
+      <c r="Q68" s="8" t="n"/>
+      <c r="R68" s="8" t="n"/>
+      <c r="S68" s="8" t="n"/>
+      <c r="T68" s="8" t="n"/>
+      <c r="U68" s="8" t="n"/>
+      <c r="V68" s="8" t="n"/>
+      <c r="W68" s="8" t="n"/>
+      <c r="X68" s="8" t="n"/>
     </row>
     <row r="69"/>
     <row r="70">
-      <c r="A70" s="20" t="inlineStr">
+      <c r="A70" s="21" t="inlineStr">
         <is>
           <t>Open-Ended AI Selection</t>
         </is>
       </c>
-      <c r="B70" s="21" t="n">
-        <v>2.52</v>
-      </c>
-      <c r="C70" s="21" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="D70" s="21" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="E70" s="21" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="F70" s="21" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="G70" s="21" t="n">
-        <v>1.055</v>
-      </c>
-      <c r="H70" s="21" t="n">
-        <v>1.035</v>
-      </c>
-      <c r="I70" s="21" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="J70" s="21" t="n">
-        <v>1.015</v>
-      </c>
-      <c r="K70" s="21" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="L70" s="21" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="M70" s="21" t="n">
-        <v>1.005</v>
-      </c>
-      <c r="N70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="O70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="P70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="R70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="S70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="T70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="U70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="V70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="W70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="X70" s="21" t="n">
-        <v>1</v>
-      </c>
+      <c r="B70" s="22" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="C70" s="22" t="n">
+        <v>1.1916</v>
+      </c>
+      <c r="D70" s="22" t="n">
+        <v>1.1507</v>
+      </c>
+      <c r="E70" s="22" t="n">
+        <v>1.0512</v>
+      </c>
+      <c r="F70" s="22" t="n">
+        <v>1.0569</v>
+      </c>
+      <c r="G70" s="22" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="H70" s="22" t="n">
+        <v>1.0153</v>
+      </c>
+      <c r="I70" s="22" t="n">
+        <v>1.0152</v>
+      </c>
+      <c r="J70" s="22" t="n">
+        <v>1.0228</v>
+      </c>
+      <c r="K70" s="22" t="n">
+        <v>1.0114</v>
+      </c>
+      <c r="L70" s="22" t="n">
+        <v>1.0242</v>
+      </c>
+      <c r="M70" s="22" t="n">
+        <v>1.004</v>
+      </c>
+      <c r="N70" s="22" t="n">
+        <v>1.0039</v>
+      </c>
+      <c r="O70" s="22" t="n">
+        <v>1.0075</v>
+      </c>
+      <c r="P70" s="22" t="n">
+        <v>1.006</v>
+      </c>
+      <c r="Q70" s="22" t="n">
+        <v>1.0114</v>
+      </c>
+      <c r="R70" s="22" t="n">
+        <v>1.0022</v>
+      </c>
+      <c r="S70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="T70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="U70" s="22" t="n">
+        <v>1.0139</v>
+      </c>
+      <c r="V70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="W70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="X70" s="23" t="n"/>
     </row>
     <row r="71" ht="60" customHeight="1">
-      <c r="A71" s="20" t="inlineStr">
+      <c r="A71" s="21" t="inlineStr">
         <is>
           <t>Open-Ended AI Reasoning</t>
         </is>
       </c>
-      <c r="B71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 2.52 from recent year consensus (2019-2023: 2.67, 2.55, 2.00, 2.46, 3.28). Pattern mirrors paid loss with slight elevation. Trimmed mean of 2015-2023 is ~2.5-2.55, accounting for 2023 outlier at 3.28.</t>
-        </is>
-      </c>
-      <c r="C71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.40 from recent mean (2019-2023: 1.76, 1.19, 1.68, 1.07, 1.60). Similar to paid loss with slight upward adjustment reflecting incurred nature.</t>
-        </is>
-      </c>
-      <c r="D71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.17 from recent consensus (2019-2023: 1.19, 1.13, 1.09, 1.21, 1.07). Slightly elevated vs paid loss due to incurred claims settling and reopening.</t>
-        </is>
-      </c>
-      <c r="E71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.12 from recent sample (2019-2023: 1.24, 1.03, 1.09, 1.02, 1.09). Incurred shows slightly more development than paid at this interval.</t>
-        </is>
-      </c>
-      <c r="F71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.07 from recent mean (2019-2023: 1.23, 1.02, 1.06, 1.08, 1.05). Modest tail development continues.</t>
-        </is>
-      </c>
-      <c r="G71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.055 from recent range (2019-2023: 1.23, 1.06, 1.06, 1.06, 1.05). Slow development.</t>
-        </is>
-      </c>
-      <c r="H71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.035 from recent mean (2019-2023: 1.06, 1.05, 1.04, 1.05, 1.04). Very low tail development.</t>
-        </is>
-      </c>
-      <c r="I71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.02 from recent pattern (2019-2023: 1.05, 1.04, 1.02, 1.04, 1.02).</t>
-        </is>
-      </c>
-      <c r="J71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.015 from recent mean near 1.01-1.015.</t>
-        </is>
-      </c>
-      <c r="K71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.01 from recent consolidation.</t>
-        </is>
-      </c>
-      <c r="L71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.01 from tail pattern.</t>
-        </is>
-      </c>
-      <c r="M71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.005 from tail development approaching zero.</t>
-        </is>
-      </c>
-      <c r="N71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 from mature tail.</t>
-        </is>
-      </c>
-      <c r="O71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="P71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="Q71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="R71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="S71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="T71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="U71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="V71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="W71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="X71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
+      <c r="B71" s="24" t="inlineStr">
+        <is>
+          <t>Early development shows strong variability (CV_10yr=0.27). Simple average is 1.7774 but benefits from trimming outliers due to 2015/2018 spikes. Weighted average (1.7371) balances recent stability with historical development. Selected 1.68 slightly below weighted 10yr, recognizing recent accounts (2022-2024) show more modest development around 1.23-1.41 range, suggesting pattern may be moderating.</t>
+        </is>
+      </c>
+      <c r="C71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.1768 suggests reasonable stability. Age-to-age factors range from 0.97 to 1.51. Simple 10yr average 1.2539, weighted 10yr 1.2877. Trimmed average (exclude high/low) at 1.2525 is more conservative. Selected 1.1916 below simple average due to: (1) trend toward lower values in recent years (2024 shows 1.6941, 2023 shows 1.1), and (2) recent development pattern suggesting completion nearer early estimates.</t>
+        </is>
+      </c>
+      <c r="D71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.1051 indicates good stability. Weighted 10yr average 1.1886, simple 10yr 1.1801, trimmed (exclude high/low) 1.1727. Selected 1.1507 (exclude high/low all) recognizing outlier years (2018 at 1.3883, 2019 at 1.1497). Development in this interval is relatively predictable with low variance.</t>
+        </is>
+      </c>
+      <c r="E71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0465 shows strong stability. All averages cluster tightly: simple 10yr=1.0530, weighted 10yr=1.0574, trimmed=1.0491. Recent years (2020-2024) average 1.0097. Selected 1.0512 from exclude high/low all method due to presence of outliers (2015 at 1.1059, 2016 at 1.1423). Development pattern is stable, approaching closure.</t>
+        </is>
+      </c>
+      <c r="F71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0719, moderate variability. Simple 10yr=1.0646, weighted 10yr=1.0752, exclude high/low 10yr=1.0543. Data shows outliers (2007 at 1.1938, 2015 at 1.1362). Selected 1.0569 (exclude high/low all) as balanced estimate removing extreme observations. Recent development (2020-2024) around 1.01-1.03 suggests slightly lower trend.</t>
+        </is>
+      </c>
+      <c r="G71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0599, reasonable stability. Simple 10yr=1.0554, weighted 10yr=1.0671, exclude high/low 10yr=1.0537. Outliers present (2007 at 1.0636, 2015 at 1.1399). Selected 1.0372 (exclude high/low all) acknowledging trim removes highs and reflects typical behavior. Development slowing but meaningful.</t>
+        </is>
+      </c>
+      <c r="H71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0442, low variability. Simple 10yr=1.0248, weighted 10yr=1.0177, exclude high/low 10yr=1.0130. Recent years (2020-2024) show development around 1.01. Selected 1.0153 (exclude high/low all) as conservative middle ground. Data is stable; development is modest.</t>
+        </is>
+      </c>
+      <c r="I71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0266, low variability. Simple 10yr=1.0190, weighted 10yr=1.0231, exclude high/low 10yr=1.0154. All methods tightly clustered. Selected 1.0152 (exclude high/low all). Very minor development; data is consistent across years.</t>
+        </is>
+      </c>
+      <c r="J71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0374, low variability. Simple 10yr=1.0351, weighted 10yr=1.0519, exclude high/low 10yr=1.0312. Selected 1.0228 (simple 3yr=1.0389, weighted 3yr=1.0629) blending recent 3yr (1.0389) and excluding high/low to avoid 2015 (1.0962). Modest tail development.</t>
+        </is>
+      </c>
+      <c r="K71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0262, very low variability. Simple 10yr=1.0160, weighted 10yr=1.0194, exclude high/low 10yr=1.0105. Selected 1.0114 (exclude high/low all). Minimal variation across years; development largely complete.</t>
+        </is>
+      </c>
+      <c r="L71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0610, moderate variability. Simple 10yr=1.0387, weighted 10yr=1.0395, exclude high/low 10yr=1.0274. Outlier at 2012 (1.1790). Selected 1.0242 (exclude high/low all) as conservative trim estimate. Development shows some tail activity but increasingly flat.</t>
+        </is>
+      </c>
+      <c r="M71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0142, very low variability. Simple 10yr=1.0056, weighted 10yr=1.0066, exclude high/low 10yr=1.0050. All methods show near-unity development. Selected 1.0040 (exclude high/low all). Minimal tail development; approaching ultimate.</t>
+        </is>
+      </c>
+      <c r="N71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0147, very low variability. Simple 10yr=1.0034, weighted 10yr=1.0030, exclude high/low 10yr=1.0015. Selected 1.0039 (exclude high/low all). Very flat development; data is highly stable.</t>
+        </is>
+      </c>
+      <c r="O71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0146, very low variability. Simple 10yr=1.0104, weighted 10yr=1.0167, exclude high/low 10yr=1.0075. Selected 1.0075 (exclude high/low all). Minor tail development; reflects data consensus.</t>
+        </is>
+      </c>
+      <c r="P71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0166, low variability. Simple 10yr=1.0106, weighted 10yr=1.0116, exclude high/low 10yr=1.0060. Selected 1.0060 (exclude high/low all). Marginal development; data highly clustered.</t>
+        </is>
+      </c>
+      <c r="Q71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0175, low variability. Simple 10yr=1.0152, weighted 10yr=1.0149, exclude high/low 10yr=1.0114. Selected 1.0114 (exclude high/low all). Slight uptick in factors; reasonable balance across estimation methods.</t>
+        </is>
+      </c>
+      <c r="R71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0112, very low variability. Simple 10yr=1.0060, weighted 10yr=1.0069, exclude high/low 10yr=1.0022. Selected 1.0022 (exclude high/low all). Minimal development; triangle nearing completion.</t>
+        </is>
+      </c>
+      <c r="S71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0073, extremely low variability. All recent years show 1.0 or near-1.0. Simple 10yr=1.0030, exclude high/low 10yr=1.0000. Selected 1.0000 reflecting data consensus and marginal/zero development in this tail interval.</t>
+        </is>
+      </c>
+      <c r="T71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0188, low variability but with some outliers (2015 at 1.0962). Simple 10yr=1.0085, weighted 10yr=1.0089, exclude high/low 10yr=1.0000. Selected 1.0000 (exclude high/low all) reflecting majority of years showing zero/negligible development.</t>
+        </is>
+      </c>
+      <c r="U71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0130, very low variability. Simple 10yr=1.0166, weighted 10yr=1.0174, exclude high/low 10yr=1.0139. Selected 1.0139 (exclude high/low all). Minor tail development; age approaching 250 months (20+ years).</t>
+        </is>
+      </c>
+      <c r="V71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0178, extremely sparse data (only 2022-2024 with values). Simple 10yr=1.0166, weighted 10yr=1.0174, exclude high/low 10yr=1.0139. Selected 1.0000 reflecting deep-tail plateau. Development essentially complete.</t>
+        </is>
+      </c>
+      <c r="W71" s="24" t="inlineStr">
+        <is>
+          <t>CV_10yr=0.0000, no variation in available data. All averages including simple, weighted show 1.0000. Selected 1.0000. Minimal observations; triangle effectively closed.</t>
+        </is>
+      </c>
+      <c r="X71" s="24" t="inlineStr">
+        <is>
+          <t>[CUTOFF] Cutoff at 263: Beyond 263 months (21+ years), data becomes too sparse and triangular development is largely complete. Very old cohorts with minimal incremental loss activity. Recommend tail curve fitting (exponential or power-law) for any extrapolation beyond this cutoff rather than direct factor selection.</t>
         </is>
       </c>
     </row>
     <row r="72"/>
     <row r="73">
-      <c r="A73" s="23" t="inlineStr">
+      <c r="A73" s="25" t="inlineStr">
         <is>
           <t>User Selection</t>
         </is>
       </c>
-      <c r="B73" s="24" t="n"/>
-      <c r="C73" s="24" t="n"/>
-      <c r="D73" s="24" t="n"/>
-      <c r="E73" s="24" t="n"/>
-      <c r="F73" s="24" t="n"/>
-      <c r="G73" s="24" t="n"/>
-      <c r="H73" s="24" t="n"/>
-      <c r="I73" s="24" t="n"/>
-      <c r="J73" s="24" t="n"/>
-      <c r="K73" s="24" t="n"/>
-      <c r="L73" s="24" t="n"/>
-      <c r="M73" s="24" t="n"/>
-      <c r="N73" s="24" t="n"/>
-      <c r="O73" s="24" t="n"/>
-      <c r="P73" s="24" t="n"/>
-      <c r="Q73" s="24" t="n"/>
-      <c r="R73" s="24" t="n"/>
-      <c r="S73" s="24" t="n"/>
-      <c r="T73" s="24" t="n"/>
-      <c r="U73" s="24" t="n"/>
-      <c r="V73" s="24" t="n"/>
-      <c r="W73" s="24" t="n"/>
-      <c r="X73" s="24" t="n"/>
+      <c r="B73" s="26" t="n"/>
+      <c r="C73" s="26" t="n"/>
+      <c r="D73" s="26" t="n"/>
+      <c r="E73" s="26" t="n"/>
+      <c r="F73" s="26" t="n"/>
+      <c r="G73" s="26" t="n"/>
+      <c r="H73" s="26" t="n"/>
+      <c r="I73" s="26" t="n"/>
+      <c r="J73" s="26" t="n"/>
+      <c r="K73" s="26" t="n"/>
+      <c r="L73" s="26" t="n"/>
+      <c r="M73" s="26" t="n"/>
+      <c r="N73" s="26" t="n"/>
+      <c r="O73" s="26" t="n"/>
+      <c r="P73" s="26" t="n"/>
+      <c r="Q73" s="26" t="n"/>
+      <c r="R73" s="26" t="n"/>
+      <c r="S73" s="26" t="n"/>
+      <c r="T73" s="26" t="n"/>
+      <c r="U73" s="26" t="n"/>
+      <c r="V73" s="26" t="n"/>
+      <c r="W73" s="26" t="n"/>
+      <c r="X73" s="26" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="23" t="inlineStr">
+      <c r="A74" s="25" t="inlineStr">
         <is>
           <t>User Reasoning</t>
         </is>
@@ -7741,74 +7677,52 @@
         </is>
       </c>
       <c r="B67" s="18" t="n">
-        <v>2.6232</v>
+        <v>2.4566</v>
       </c>
       <c r="C67" s="18" t="n">
-        <v>1.4224</v>
+        <v>1.3437</v>
       </c>
       <c r="D67" s="18" t="n">
-        <v>1.1663</v>
+        <v>1.1803</v>
       </c>
       <c r="E67" s="18" t="n">
-        <v>1.103</v>
+        <v>1.1038</v>
       </c>
       <c r="F67" s="18" t="n">
-        <v>1.1239</v>
+        <v>1.0774</v>
       </c>
       <c r="G67" s="18" t="n">
-        <v>1.1184</v>
+        <v>1.0591</v>
       </c>
       <c r="H67" s="18" t="n">
-        <v>1.0377</v>
+        <v>1.026</v>
       </c>
       <c r="I67" s="18" t="n">
-        <v>1.0124</v>
+        <v>1.0208</v>
       </c>
       <c r="J67" s="18" t="n">
-        <v>1.0814</v>
+        <v>1.0394</v>
       </c>
       <c r="K67" s="18" t="n">
-        <v>1.0108</v>
+        <v>1.0282</v>
       </c>
       <c r="L67" s="18" t="n">
-        <v>1.0204</v>
+        <v>1.0226</v>
       </c>
       <c r="M67" s="18" t="n">
-        <v>1.0156</v>
-      </c>
-      <c r="N67" s="18" t="n">
-        <v>1.0075</v>
-      </c>
-      <c r="O67" s="18" t="n">
-        <v>1.0083</v>
-      </c>
-      <c r="P67" s="18" t="n">
-        <v>1.0175</v>
-      </c>
-      <c r="Q67" s="18" t="n">
-        <v>1.0112</v>
-      </c>
-      <c r="R67" s="18" t="n">
-        <v>1.0025</v>
-      </c>
-      <c r="S67" s="18" t="n">
-        <v>1.0032</v>
-      </c>
-      <c r="T67" s="18" t="n">
-        <v>1.0012</v>
-      </c>
-      <c r="U67" s="18" t="n">
-        <v>1.0049</v>
-      </c>
-      <c r="V67" s="18" t="n">
-        <v>1.0062</v>
-      </c>
-      <c r="W67" s="18" t="n">
-        <v>1.0074</v>
-      </c>
-      <c r="X67" s="18" t="n">
-        <v>1.0039</v>
-      </c>
+        <v>1.0211</v>
+      </c>
+      <c r="N67" s="19" t="n"/>
+      <c r="O67" s="19" t="n"/>
+      <c r="P67" s="19" t="n"/>
+      <c r="Q67" s="19" t="n"/>
+      <c r="R67" s="19" t="n"/>
+      <c r="S67" s="19" t="n"/>
+      <c r="T67" s="19" t="n"/>
+      <c r="U67" s="19" t="n"/>
+      <c r="V67" s="19" t="n"/>
+      <c r="W67" s="19" t="n"/>
+      <c r="X67" s="19" t="n"/>
     </row>
     <row r="68" ht="60" customHeight="1">
       <c r="A68" s="17" t="inlineStr">
@@ -7816,354 +7730,312 @@
           <t>Rules-Based AI Reasoning</t>
         </is>
       </c>
-      <c r="B68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: 5-year volume-weighted average: standard selection for paid loss.</t>
-        </is>
-      </c>
-      <c r="C68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Downward trend in paid detected. Conservative: held at 5-year; paid loss patterns less volatile than incurred.</t>
-        </is>
-      </c>
-      <c r="D68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0502) and 5yr (0.1004); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="E68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.1057) and 5yr (0.0759); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="F68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0721) and 5yr (0.0522); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="G68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.1012) and 5yr (0.0961); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="H68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0403) and 5yr (0.0391); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="I68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0040) and 5yr (0.0112); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="J68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0647) and 5yr (0.0566); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="K68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0153) and 5yr (0.0121); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="L68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0294) and 5yr (0.0237); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="M68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0226) and 5yr (0.0235); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="N68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0017) and 5yr (0.0123); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="O68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0033) and 5yr (0.0108); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="P68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0159) and 5yr (0.0114); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="Q68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0103) and 5yr (0.0103); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="R68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0033) and 5yr (0.0031); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="S68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0032) and 5yr (0.0069); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="T68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0000) and 5yr (0.0054); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="U68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0058) and 5yr (0.0051); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="V68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0050) and 5yr (0.0050); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="W68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: Low variability on both 3yr (0.0019) and 5yr (0.0019); averages stable and credible. Used 50/50 blend of 3yr/5yr for balance.</t>
-        </is>
-      </c>
-      <c r="X68" s="19" t="inlineStr">
-        <is>
-          <t>Paid Loss: 5-year volume-weighted average: standard selection for paid loss.</t>
-        </is>
-      </c>
+      <c r="B68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 2.4566. CV_5yr = 0.1774 (within 0.10-0.20 range requiring outlier handling). All averages converge within 4% (simple_5yr: 2.5842, weighted_5yr: 2.4566, avg_exclude_high_low_5yr: 2.5525), supporting selection from core convergent band. Strong positive 3-year slope (0.6336) indicates recent acceleration; 5-year slope positive (0.1057) suggests sustained upward trend likely due to inflation. No diagnostic contradictions. Weighted approach balances large-AY dominance while capturing recent acceleration.</t>
+        </is>
+      </c>
+      <c r="C68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.3437. CV_5yr = 0.2103 (&gt;0.10, outlier exclusion applied). Exclude high/low average = 1.3321, close to weighted (1.3437) confirming central tendency. Simple 5-year = 1.4224 is 4.7% above, triggering Bayesian check. Positive 3yr slope (offset by negative 5yr slope) suggests recent stabilization rather than trend. Maturity-dependent: at 23-35mo (early), maintain 5-year window. Selection reflects conservative approach with slight upward bias from weighted scheme.</t>
+        </is>
+      </c>
+      <c r="D68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.1803. CV_5yr = 0.1004 (within acceptable range). All averages tightly clustered (simple_5yr: 1.1749, avg_exclude_high_low_5yr: 1.1638), confirming convergence within ±1%. Data quality excellent. No slope signal (5yr = -0.0368). Early maturity (35-47mo): 5-year window appropriate. Selection reflects strongest convergence zone with minimal volatility.</t>
+        </is>
+      </c>
+      <c r="E68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.1038. CV_5yr = 0.0759 (low, &lt;0.10). Convergence: simple_5yr = 1.0924, weighted = 1.1038, exclude_high_low = 1.0734, all within ±2% of weighted. Slope stable (5yr = 0.0014, near-zero). Transition from early to mid-maturity (47-59mo); 5-year window justified by consistent pattern. Selection balances volume weighting with data credibility.</t>
+        </is>
+      </c>
+      <c r="F68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0774. CV_5yr = 0.0522 (low). All averages converge tightly (simple_5yr: 1.1190, weighted: 1.0774, exclude: not significantly different), within ±2%. Positive 5yr slope = 0.0158 suggests gentle upward trend, likely inflation-related; 3yr slope = 0.0539 higher, indicating acceleration. Mid-maturity (59-71mo): 5-year sufficient for pattern. No asymmetric conservatism adjustment needed given tight convergence. Selection reflects stable development with mild inflation signal.</t>
+        </is>
+      </c>
+      <c r="G68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0591. CV_5yr = 0.0961 (elevated but &lt;0.15). All averages within ±3% (simple_5yr: 1.1215, weighted: 1.0591, exclude_high_low: 1.1033), confirming central convergence despite higher variance. Slope data: 5yr = 0.0287, 3yr = -0.04 (conflicting signals, 3yr less reliable). At 71-83mo (mid-late maturity), larger volume weight justifies variance absorption. No external diagnostics override. Selection uses weighted approach to anchor to larger AYs.</t>
+        </is>
+      </c>
+      <c r="H68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0260. CV_5yr = 0.0391 (very low). Convergence excellent: simple_5yr = 1.0311, weighted = 1.0260, exclude_high_low = 1.0214, all within ±1.5%. Slope nearly zero (5yr = 0.0186, 3yr = 0.0182). Late maturity (83-95mo): development stable. Minimal outlier influence. Selection reflects high-credibility zone with tight clustering across all methods.</t>
+        </is>
+      </c>
+      <c r="I68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0208. CV_5yr = 0.0112 (extremely low). Convergence perfect: all averages within ±2% of weighted. Slope minimal (5yr = -0.0028, near-zero). Late maturity (95-107mo): data minimal but consistent. Weighted approach maintains rigor despite sparse diagonal. Selection represents stable tail development with near-zero variance.</t>
+        </is>
+      </c>
+      <c r="J68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0394. CV_5yr = 0.0566 (moderate). All averages converge within ±3% (simple_5yr: 1.0423, weighted: 1.0394, exclude_high_low: 1.0246). Positive 5yr slope = 0.0317 consistent with 3yr = 0.0689, indicating continued development acceleration (possibly late-stage frequency effects or case reopenings). Late maturity (107-119mo): 5-year window appropriate despite sparse data. Selection anchors to weighted while acknowledging upward trend signal.</t>
+        </is>
+      </c>
+      <c r="K68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0282. CV_5yr = 0.0121 (very low). Convergence: simple_5yr = 1.0086, weighted = 1.0282, exclude_high_low = 1.0044, range ±2.5%. Slope stable (5yr = 0.0009, minimal). Late maturity (119-131mo): consistent, credible development. Selection uses weighted to stabilize sparse data while remaining realistic. No material diagnostic impact.</t>
+        </is>
+      </c>
+      <c r="L68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0226. CV_5yr = 0.0237 (very low). All averages within ±2% (simple_5yr: 1.0195, weighted: 1.0226, exclude_high_low: 1.0136). Slope negligible (5yr = -0.0005). Very late maturity (131-143mo): sparse data, but pattern consistent. Selection uses weighted for rigor. Development slowing as expected at this tail point.</t>
+        </is>
+      </c>
+      <c r="M68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0211. CV_5yr = 0.0235 (very low). Convergence tight: simple_5yr = 1.0201, weighted = 1.0211, exclude_high_low = 1.0167, all within ±1.5%. Slope minimal (5yr = 0.0036). Very late maturity (143-155mo): extremely sparse data, but consistent across methods. Last credible LDF with meaningful development signal. Selection supports tail factoring from this point onward.</t>
+        </is>
+      </c>
+      <c r="N68" s="20" t="inlineStr">
+        <is>
+          <t>[CUTOFF] CUTOFF at 155 months: is_monotone_from_here = expected True from sparse pattern; CV from 155+ averages = 0.0123 (low); slope_sign_changes = 0 (stable direction). 5 factors minimum for curve fit available from 155-287 (5 intervals). Rejection rationale: Data extremely sparse beyond 155 months with only 2-3 AY diagonals per column. Paid loss at 155+mo represents tail beyond typical development window (paid loss minimum cutoff: 60mo, exceeded). Switching to tail curve methodology for 155+mo intervals ensures stability and prevents overfitting. Latest diagonal factors at 143-155 show minimal development (LDF=1.0211), consistent with end-of-development signal.</t>
+        </is>
+      </c>
+      <c r="O68" s="8" t="n"/>
+      <c r="P68" s="8" t="n"/>
+      <c r="Q68" s="8" t="n"/>
+      <c r="R68" s="8" t="n"/>
+      <c r="S68" s="8" t="n"/>
+      <c r="T68" s="8" t="n"/>
+      <c r="U68" s="8" t="n"/>
+      <c r="V68" s="8" t="n"/>
+      <c r="W68" s="8" t="n"/>
+      <c r="X68" s="8" t="n"/>
     </row>
     <row r="69"/>
     <row r="70">
-      <c r="A70" s="20" t="inlineStr">
+      <c r="A70" s="21" t="inlineStr">
         <is>
           <t>Open-Ended AI Selection</t>
         </is>
       </c>
-      <c r="B70" s="21" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="C70" s="21" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="D70" s="21" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="E70" s="21" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="F70" s="21" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="G70" s="21" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="H70" s="21" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="I70" s="21" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="J70" s="21" t="n">
+      <c r="B70" s="22" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="C70" s="22" t="n">
+        <v>1.3321</v>
+      </c>
+      <c r="D70" s="22" t="n">
+        <v>1.1638</v>
+      </c>
+      <c r="E70" s="22" t="n">
+        <v>1.0987</v>
+      </c>
+      <c r="F70" s="22" t="n">
+        <v>1.0618</v>
+      </c>
+      <c r="G70" s="22" t="n">
+        <v>1.0456</v>
+      </c>
+      <c r="H70" s="22" t="n">
+        <v>1.0203</v>
+      </c>
+      <c r="I70" s="22" t="n">
         <v>1.015</v>
       </c>
-      <c r="K70" s="21" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="L70" s="21" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="M70" s="21" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="N70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="O70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="P70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="R70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="S70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="T70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="U70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="V70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="W70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="X70" s="21" t="n">
-        <v>1</v>
-      </c>
+      <c r="J70" s="22" t="n">
+        <v>1.0219</v>
+      </c>
+      <c r="K70" s="22" t="n">
+        <v>1.0182</v>
+      </c>
+      <c r="L70" s="22" t="n">
+        <v>1.0173</v>
+      </c>
+      <c r="M70" s="22" t="n">
+        <v>1.0174</v>
+      </c>
+      <c r="N70" s="22" t="n">
+        <v>1.0106</v>
+      </c>
+      <c r="O70" s="22" t="n">
+        <v>1.0104</v>
+      </c>
+      <c r="P70" s="22" t="n">
+        <v>1.011</v>
+      </c>
+      <c r="Q70" s="22" t="n">
+        <v>1.0157</v>
+      </c>
+      <c r="R70" s="22" t="n">
+        <v>1.0063</v>
+      </c>
+      <c r="S70" s="22" t="n">
+        <v>1.0054</v>
+      </c>
+      <c r="T70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="U70" s="22" t="n">
+        <v>1.0037</v>
+      </c>
+      <c r="V70" s="22" t="n">
+        <v>1.0074</v>
+      </c>
+      <c r="W70" s="22" t="n">
+        <v>1.0076</v>
+      </c>
+      <c r="X70" s="23" t="n"/>
     </row>
     <row r="71" ht="60" customHeight="1">
-      <c r="A71" s="20" t="inlineStr">
+      <c r="A71" s="21" t="inlineStr">
         <is>
           <t>Open-Ended AI Reasoning</t>
         </is>
       </c>
-      <c r="B71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 2.50 based on recent year pattern (2019-2023: 2.67, 2.55, 1.99, 2.43, 3.27). Recent years show volatility around 2.5-2.7, but excluding extreme 3.27 outlier from 2023 and 1.79 from 2014, the centroid of 2015-2022 is ~2.5. This represents strong early development typical of this account but acknowledges normalization in recent cohorts.</t>
-        </is>
-      </c>
-      <c r="C71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.38 from robust recent year consensus (2019-2023: 1.75, 1.18, 1.67, 1.06, 1.59). Trimmed average of last 10 years (excluding extremes) centers around 1.35-1.40. This interval shows consistent, credible development with less volatility than 11-23.</t>
-        </is>
-      </c>
-      <c r="D71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.15 from recent period average (2019-2023: 1.18, 1.12, 1.07, 1.19, 1.06). The last decade averages 1.12-1.15 with stable pattern. This interval shows moderate tail development.</t>
-        </is>
-      </c>
-      <c r="E71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.10 based on 2015-2023 mean of ~1.09-1.12. Recent years show tight clustering: 1.23, 1.01, 1.07, 1.01, 1.07. Reflects modest development at this maturity.</t>
-        </is>
-      </c>
-      <c r="F71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.06 from recent consensus (2019-2023: 1.22, 1.01, 1.05, 1.07, 1.04). Last decade averages 1.055-1.065. Development continues to slow.</t>
-        </is>
-      </c>
-      <c r="G71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.05 based on recent years (2019-2023: 1.22, 1.05, 1.05, 1.05, 1.04) and broader sample showing range 1.00-1.14. Pattern suggests slight tail development continues.</t>
-        </is>
-      </c>
-      <c r="H71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.03 from recent mean (2019-2023: 1.05, 1.04, 1.03, 1.04, 1.04). Very stable interval with minimal tail development.</t>
-        </is>
-      </c>
-      <c r="I71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.02 from recent years (2019-2023: 1.04, 1.03, 1.01, 1.03, 1.01). Consistent low development.</t>
-        </is>
-      </c>
-      <c r="J71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.015 from tight recent range (2019-2023: 1.01, 1.00, 1.01, 1.00, 1.04). Minimal development at advanced maturity.</t>
-        </is>
-      </c>
-      <c r="K71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.01 from recent cluster (2019-2023: 1.01, 1.01, 1.01, 1.01, 1.04). Very minimal tail development.</t>
-        </is>
-      </c>
-      <c r="L71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.01 based on recent years averaging near 1.01-1.02 with many factors at exactly 1.00 or very close.</t>
-        </is>
-      </c>
-      <c r="M71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.01 from recent pattern showing development near 1.00-1.01 range.</t>
-        </is>
-      </c>
-      <c r="N71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 as recent years show factors clustering at or very near 1.00, indicating maturity.</t>
-        </is>
-      </c>
-      <c r="O71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 from consolidated tail factors approaching ultimate.</t>
-        </is>
-      </c>
-      <c r="P71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 as tail development is minimal.</t>
-        </is>
-      </c>
-      <c r="Q71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 from tail consolidation.</t>
-        </is>
-      </c>
-      <c r="R71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for very long tail, assuming near-ultimate.</t>
-        </is>
-      </c>
-      <c r="S71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for far tail.</t>
-        </is>
-      </c>
-      <c r="T71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for far tail.</t>
-        </is>
-      </c>
-      <c r="U71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for far tail.</t>
-        </is>
-      </c>
-      <c r="V71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for far tail.</t>
-        </is>
-      </c>
-      <c r="W71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for far tail.</t>
-        </is>
-      </c>
-      <c r="X71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for far tail.</t>
+      <c r="B71" s="24" t="inlineStr">
+        <is>
+          <t>Highly volatile early development (CV_10yr=0.2259). Simple 10yr=2.4862, weighted 10yr=2.4820, exclude high/low 10yr=2.4762. All averages cluster around 2.48. Selected 2.4000 slightly conservative due to: (1) 2024 shows 1.6941 suggesting recent slowdown, (2) slope analysis shows negative 5yr/10yr trend, (3) 2022-2024 trend averaging ~1.5-1.7 suggests development pattern moderating. Conservative selection accounts for possible economic/underwriting changes.</t>
+        </is>
+      </c>
+      <c r="C71" s="24" t="inlineStr">
+        <is>
+          <t>Moderate variability (CV_10yr=0.1904). Simple 10yr=1.3735, weighted 10yr=1.3913, exclude high/low 10yr=1.3658. Selected 1.3321 (exclude high/low all) recognizing outliers and reflecting conservative trim estimate. Data shows this interval captures key development; trend analysis (slope_10yr=0.0049) shows minimal directional bias.</t>
+        </is>
+      </c>
+      <c r="D71" s="24" t="inlineStr">
+        <is>
+          <t>Low-to-moderate variability (CV_10yr=0.1076). Simple 10yr=1.2026, weighted 10yr=1.2249, exclude high/low 10yr=1.1864. Selected 1.1638 (exclude high/low all) as balanced conservative estimate. Age-to-age factors show range 1.04-1.39 with outliers. Trim removes extremes (2015 at 1.3285, 2019 at 1.1497) for stable middle ground.</t>
+        </is>
+      </c>
+      <c r="E71" s="24" t="inlineStr">
+        <is>
+          <t>Moderate variability (CV_10yr=0.0642). Simple 10yr=1.0882, weighted 10yr=1.0874, exclude high/low 10yr=1.0800. Selected 1.0987 (simple 5yr=1.0924) reflecting recent trend. Development meaningful; 2007 shows 1.1147 (outlier), 2015 shows 1.1059. Selection balances recent data with longer history.</t>
+        </is>
+      </c>
+      <c r="F71" s="24" t="inlineStr">
+        <is>
+          <t>Low-moderate variability (CV_10yr=0.0625). Simple 10yr=1.0725, weighted 10yr=1.0861, exclude high/low 10yr=1.0640. Selected 1.0618 (exclude high/low all) as conservative trim. Outliers present (2007 at 1.1938, 2015 at 1.1362). Development moderating; data shows clustering near 1.02-1.07.</t>
+        </is>
+      </c>
+      <c r="G71" s="24" t="inlineStr">
+        <is>
+          <t>Low variability (CV_10yr=0.0817). Simple 10yr=1.0796, weighted 10yr=1.0846, exclude high/low 10yr=1.0630. Selected 1.0456 (exclude high/low all) recognizing outliers (2007 at 1.0636, 2015 at 1.1275, 2019 at 1.2221). Conservative trim estimate. Meaningful tail development continues.</t>
+        </is>
+      </c>
+      <c r="H71" s="24" t="inlineStr">
+        <is>
+          <t>Low-moderate variability (CV_10yr=0.0308). Simple 10yr=1.0255, weighted 10yr=1.0256, exclude high/low 10yr=1.0205. Selected 1.0203 (exclude high/low all). Age-to-age factors show range 0.98-1.24 with sparse high observations. Development slowing; approaching practical tail.</t>
+        </is>
+      </c>
+      <c r="I71" s="24" t="inlineStr">
+        <is>
+          <t>Very low variability (CV_10yr=0.0238). Simple 10yr=1.0202, weighted 10yr=1.0254, exclude high/low 10yr=1.0150. Selected 1.0150 (exclude high/low all). Minimal, predictable development. Recent years (2020-2024) average 1.0-1.05. Marginal tail development.</t>
+        </is>
+      </c>
+      <c r="J71" s="24" t="inlineStr">
+        <is>
+          <t>Low variability (CV_10yr=0.0440). Simple 10yr=1.0366, weighted 10yr=1.0547, exclude high/low 10yr=1.0286. Selected 1.0219 (simple 3yr=1.0665, weighted 3yr=1.0982, recent bias toward 1.03-1.10). Moderate tail factor; selection blends recent behavior with conservative estimate.</t>
+        </is>
+      </c>
+      <c r="K71" s="24" t="inlineStr">
+        <is>
+          <t>Low variability (CV_10yr=0.0327). Simple 10yr=1.0266, weighted 10yr=1.0353, exclude high/low 10yr=1.0217. Selected 1.0182 (exclude high/low all). Outlier at 2012 (1.0124, modestly high). Modest tail development; age approaching 10+ years.</t>
+        </is>
+      </c>
+      <c r="L71" s="24" t="inlineStr">
+        <is>
+          <t>Low variability (CV_10yr=0.0201). Simple 10yr=1.0204, weighted 10yr=1.0254, exclude high/low 10yr=1.0184. Selected 1.0173 (exclude high/low all). All methods cluster tightly. Outlier at 2012 (1.0223) modestly high. Stable, marginal development.</t>
+        </is>
+      </c>
+      <c r="M71" s="24" t="inlineStr">
+        <is>
+          <t>Low variability (CV_10yr=0.0200). Simple 10yr=1.0185, weighted 10yr=1.0215, exclude high/low 10yr=1.0169. Selected 1.0174 (exclude high/low all). Data highly stable with little variation. Marginal tail development continuing.</t>
+        </is>
+      </c>
+      <c r="N71" s="24" t="inlineStr">
+        <is>
+          <t>Very low variability (CV_10yr=0.0116). Simple 10yr=1.0114, weighted 10yr=1.0137, exclude high/low 10yr=1.0087. Selected 1.0106 (exclude high/low all). Minimal development; nearly complete closure by age 155 months (~12.9 years).</t>
+        </is>
+      </c>
+      <c r="O71" s="24" t="inlineStr">
+        <is>
+          <t>Very low variability (CV_10yr=0.0120). Simple 10yr=1.0114, weighted 10yr=1.0156, exclude high/low 10yr=1.0104. Selected 1.0104 (exclude high/low all). Virtually flat development; consensus from all methods.</t>
+        </is>
+      </c>
+      <c r="P71" s="24" t="inlineStr">
+        <is>
+          <t>Very low variability (CV_10yr=0.0116). Simple 10yr=1.0120, weighted 10yr=1.0163, exclude high/low 10yr=1.0110. Selected 1.0110 (exclude high/low all). Extremely minor development; data stable across cohorts.</t>
+        </is>
+      </c>
+      <c r="Q71" s="24" t="inlineStr">
+        <is>
+          <t>Very low variability (CV_10yr=0.0124). Simple 10yr=1.0158, weighted 10yr=1.0158, exclude high/low 10yr=1.0157. Selected 1.0157 (exclude high/low all). Methods converge; very stable tail factor. Age ~16 years.</t>
+        </is>
+      </c>
+      <c r="R71" s="24" t="inlineStr">
+        <is>
+          <t>Very low variability (CV_10yr=0.0108). Simple 10yr=1.0084, weighted 10yr=1.0087, exclude high/low 10yr=1.0063. Selected 1.0063 (exclude high/low all). Marginal development; well into tail period.</t>
+        </is>
+      </c>
+      <c r="S71" s="24" t="inlineStr">
+        <is>
+          <t>Very low variability (CV_10yr=0.0151). Simple 10yr=1.0099, weighted 10yr=1.0130, exclude high/low 10yr=1.0054. Selected 1.0054 (exclude high/low all) as conservative trim reflecting outliers. Minimal development; practical closure imminent.</t>
+        </is>
+      </c>
+      <c r="T71" s="24" t="inlineStr">
+        <is>
+          <t>Very low variability (CV_10yr=0.0054). Simple 10yr=1.0024, weighted 10yr=1.0025, exclude high/low 10yr=1.0000. Selected 1.0000 (exclude high/low all) reflecting flat development and consensus toward unity in deep tail.</t>
+        </is>
+      </c>
+      <c r="U71" s="24" t="inlineStr">
+        <is>
+          <t>Very low variability (CV_10yr=0.0051). Simple 10yr=1.0044, weighted 10yr=1.0054, exclude high/low 10yr=1.0037. Selected 1.0037 (exclude high/low all). Marginal tail development; age ~20 years.</t>
+        </is>
+      </c>
+      <c r="V71" s="24" t="inlineStr">
+        <is>
+          <t>Very low variability (CV_10yr=0.0050). Simple 10yr=1.0057, weighted 10yr=1.0062, exclude high/low 10yr=1.0074. Selected 1.0074 (exclude high/low all). Sparse recent data (2022-2024) shows consistent ~1.006-1.008. Minor tail activity.</t>
+        </is>
+      </c>
+      <c r="W71" s="24" t="inlineStr">
+        <is>
+          <t>Very low variability (CV_10yr=0.0019). Simple 10yr=1.0076, weighted 10yr=1.0074, exclude high/low 10yr=1.0076. Selected 1.0076 (exclude high/low all). Extremely stable; all methods agree closely. Deep tail development.</t>
+        </is>
+      </c>
+      <c r="X71" s="24" t="inlineStr">
+        <is>
+          <t>[CUTOFF] Cutoff at 263: Beyond 263 months (~21+ years), data becomes extremely sparse (2024 only has 1 observation at 1.0039). Tail development is minimal and unreliable for direct selection. Recommend tail curve fitting (exponential decay model) for extrapolation beyond this point rather than factor-based selection.</t>
         </is>
       </c>
     </row>
     <row r="72"/>
     <row r="73">
-      <c r="A73" s="23" t="inlineStr">
+      <c r="A73" s="25" t="inlineStr">
         <is>
           <t>User Selection</t>
         </is>
       </c>
-      <c r="B73" s="24" t="n"/>
-      <c r="C73" s="24" t="n"/>
-      <c r="D73" s="24" t="n"/>
-      <c r="E73" s="24" t="n"/>
-      <c r="F73" s="24" t="n"/>
-      <c r="G73" s="24" t="n"/>
-      <c r="H73" s="24" t="n"/>
-      <c r="I73" s="24" t="n"/>
-      <c r="J73" s="24" t="n"/>
-      <c r="K73" s="24" t="n"/>
-      <c r="L73" s="24" t="n"/>
-      <c r="M73" s="24" t="n"/>
-      <c r="N73" s="24" t="n"/>
-      <c r="O73" s="24" t="n"/>
-      <c r="P73" s="24" t="n"/>
-      <c r="Q73" s="24" t="n"/>
-      <c r="R73" s="24" t="n"/>
-      <c r="S73" s="24" t="n"/>
-      <c r="T73" s="24" t="n"/>
-      <c r="U73" s="24" t="n"/>
-      <c r="V73" s="24" t="n"/>
-      <c r="W73" s="24" t="n"/>
-      <c r="X73" s="24" t="n"/>
+      <c r="B73" s="26" t="n"/>
+      <c r="C73" s="26" t="n"/>
+      <c r="D73" s="26" t="n"/>
+      <c r="E73" s="26" t="n"/>
+      <c r="F73" s="26" t="n"/>
+      <c r="G73" s="26" t="n"/>
+      <c r="H73" s="26" t="n"/>
+      <c r="I73" s="26" t="n"/>
+      <c r="J73" s="26" t="n"/>
+      <c r="K73" s="26" t="n"/>
+      <c r="L73" s="26" t="n"/>
+      <c r="M73" s="26" t="n"/>
+      <c r="N73" s="26" t="n"/>
+      <c r="O73" s="26" t="n"/>
+      <c r="P73" s="26" t="n"/>
+      <c r="Q73" s="26" t="n"/>
+      <c r="R73" s="26" t="n"/>
+      <c r="S73" s="26" t="n"/>
+      <c r="T73" s="26" t="n"/>
+      <c r="U73" s="26" t="n"/>
+      <c r="V73" s="26" t="n"/>
+      <c r="W73" s="26" t="n"/>
+      <c r="X73" s="26" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="23" t="inlineStr">
+      <c r="A74" s="25" t="inlineStr">
         <is>
           <t>User Reasoning</t>
         </is>
@@ -11566,74 +11438,36 @@
         </is>
       </c>
       <c r="B67" s="18" t="n">
-        <v>1.118</v>
+        <v>1.0617</v>
       </c>
       <c r="C67" s="18" t="n">
-        <v>1</v>
+        <v>1.0033</v>
       </c>
       <c r="D67" s="18" t="n">
-        <v>1.0008</v>
+        <v>1.0004</v>
       </c>
       <c r="E67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F67" s="18" t="n">
-        <v>0.9992</v>
-      </c>
-      <c r="G67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="H67" s="18" t="n">
-        <v>0.9993</v>
-      </c>
-      <c r="I67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="J67" s="18" t="n">
-        <v>0.9977</v>
-      </c>
-      <c r="K67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="L67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="M67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="N67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="O67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="P67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="R67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="S67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="T67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="U67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="V67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="W67" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="X67" s="18" t="n">
-        <v>1</v>
-      </c>
+        <v>0.9998</v>
+      </c>
+      <c r="F67" s="19" t="n"/>
+      <c r="G67" s="19" t="n"/>
+      <c r="H67" s="19" t="n"/>
+      <c r="I67" s="19" t="n"/>
+      <c r="J67" s="19" t="n"/>
+      <c r="K67" s="19" t="n"/>
+      <c r="L67" s="19" t="n"/>
+      <c r="M67" s="19" t="n"/>
+      <c r="N67" s="19" t="n"/>
+      <c r="O67" s="19" t="n"/>
+      <c r="P67" s="19" t="n"/>
+      <c r="Q67" s="19" t="n"/>
+      <c r="R67" s="19" t="n"/>
+      <c r="S67" s="19" t="n"/>
+      <c r="T67" s="19" t="n"/>
+      <c r="U67" s="19" t="n"/>
+      <c r="V67" s="19" t="n"/>
+      <c r="W67" s="19" t="n"/>
+      <c r="X67" s="19" t="n"/>
     </row>
     <row r="68" ht="60" customHeight="1">
       <c r="A68" s="17" t="inlineStr">
@@ -11641,354 +11475,280 @@
           <t>Rules-Based AI Reasoning</t>
         </is>
       </c>
-      <c r="B68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0316 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="C68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0000 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="D68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0019 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="E68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0029 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="F68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0017 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="G68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0000 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="H68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0019 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="I68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0000 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="J68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0052 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="K68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0000 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="L68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0000 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="M68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0000 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="N68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0000 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="O68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0000 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="P68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0000 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="Q68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0000 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="R68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0000 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="S68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0000 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="T68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0000 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="U68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0000 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="V68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0000 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="W68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: Very low variability: CV_5yr=0.0000 well below 0.05. 5-year average is highly credible for stable claim reporting patterns.</t>
-        </is>
-      </c>
-      <c r="X68" s="19" t="inlineStr">
-        <is>
-          <t>Reported Count: 5-year volume-weighted average: default for stable reported count development.</t>
-        </is>
-      </c>
+      <c r="B68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0617. CV_5yr = 0.0316 (very low). Convergence excellent: simple_5yr = 1.1204, weighted_5yr = 1.0617, avg_exclude_high_low_5yr = 1.1330, tight clustering with all within ±3.5%. Note: simple is 5.5% above weighted, skewed by 2016-2018 high reporters; weighted appropriately downweights this period. Slope data: 5yr = 0.0027 (near-zero), 3yr = -0.0128 (slight negative). Early maturity (11-23mo): volume weighting justified to moderate recent outlier upswing. Selection reflects convergence override principle (Section 8): multiple averages agree within ±2% of midpoint, supporting single midpoint selection.</t>
+        </is>
+      </c>
+      <c r="C68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0033. CV_5yr = 0.0000 (perfect stability). Convergence perfect: all averages = 1.0000 to 1.0069, effectively no variance. Slope minimal (5yr = -0.0 to 0.0, 3yr = 0.0). Convergence override applies (Section 8): all averages within ±1% of 1.0000-1.0069 midpoint. Selection at 1.0033 represents midpoint of converged band. Early maturity (23-35mo): count development essentially complete by 23 months post-origin. Diagnostic signals: no reported count changes year-to-year; data extremely stable. This is the tightest convergence in the entire triangle, justifying minimal LDF.</t>
+        </is>
+      </c>
+      <c r="D68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 1.0004. CV_5yr = 0.0019 (essentially zero). Convergence perfect: all averages within ±0.1% of 1.0004 (simple: 1.0005, exclude_high_low: 1.0004, weighted: 1.0004). Slope zero (5yr = -0.0002, 3yr = 0.0). Convergence override applies strongly at this interval: absolute convergence across all methods at 1.0000-1.0005 range. Selection at midpoint 1.0004. Early-to-mid maturity (35-47mo): count development near-complete. No material reporting changes in this window. Reported count triangle shows almost all AYs at same count value by 35-47 months.</t>
+        </is>
+      </c>
+      <c r="E68" s="20" t="inlineStr">
+        <is>
+          <t>Weighted 5-year LDF = 0.9998. CV_5yr = 0.0029 (extremely low). Convergence perfect: simple_5yr = 0.9999, weighted_all = 0.9998, exclude_high_low = 0.9999, all within ±0.1% of 1.0000. Slope minimal (5yr = 0.0004, 3yr = -0.002). SECTION 11 CHECK: 'Never select &lt;1.000' for paid losses, but reported counts naturally stabilize at near-1.000 as reporting completes. Selection at 0.9998 reflects true convergence around 1.000, not downward trend. Convergence override (Section 8) applies: all averages agree within ±0.15% of 1.0000 midpoint. Mid-maturity (47-59mo): this is the final meaningful development interval; counts lock at mature level. Selection reflects completion of reporting, with minimal late adjustments.</t>
+        </is>
+      </c>
+      <c r="F68" s="20" t="inlineStr">
+        <is>
+          <t>[CUTOFF] CUTOFF at 59 months (reported count): is_monotone_from_59_onward = True (all factors = 1.000 thereafter); CV_59+ = 0.0017 (near-zero); slope_sign_changes = 0. Reported count minimum type cutoff = 48 months (exceeded). Rejection rationale: (1) Data shows 100% convergence to 1.000 from 59-71 onward across all AY diagonals (values exactly 1.000 in triangle); (2) No incremental reporting occurs beyond 47-59 months (all factors = 1.0 or 1.0000 in subsequent columns); (3) Latest credible LDF at 47-59 (0.9998 ≈ 1.000) indicates reporting completion; (4) Diagnostic from triangle: reported counts plateau by 47-59 months, with zero incremental claims from 59+ onward; (5) Section 9 maturity-dependent behavior: at mid-maturity (47-59mo), transition to tail is appropriate when development stops. Convergence override applies: all averages at 59-71+ = exactly 1.000 or within ±0.001%, confirming development cessation. Switch to tail methodology for 59+mo intervals; zero tail factor (LDF=1.000) for all subsequent maturities is justified and credible.</t>
+        </is>
+      </c>
+      <c r="G68" s="8" t="n"/>
+      <c r="H68" s="8" t="n"/>
+      <c r="I68" s="8" t="n"/>
+      <c r="J68" s="8" t="n"/>
+      <c r="K68" s="8" t="n"/>
+      <c r="L68" s="8" t="n"/>
+      <c r="M68" s="8" t="n"/>
+      <c r="N68" s="8" t="n"/>
+      <c r="O68" s="8" t="n"/>
+      <c r="P68" s="8" t="n"/>
+      <c r="Q68" s="8" t="n"/>
+      <c r="R68" s="8" t="n"/>
+      <c r="S68" s="8" t="n"/>
+      <c r="T68" s="8" t="n"/>
+      <c r="U68" s="8" t="n"/>
+      <c r="V68" s="8" t="n"/>
+      <c r="W68" s="8" t="n"/>
+      <c r="X68" s="8" t="n"/>
     </row>
     <row r="69"/>
     <row r="70">
-      <c r="A70" s="20" t="inlineStr">
+      <c r="A70" s="21" t="inlineStr">
         <is>
           <t>Open-Ended AI Selection</t>
         </is>
       </c>
-      <c r="B70" s="21" t="n">
-        <v>2.35</v>
-      </c>
-      <c r="C70" s="21" t="n">
-        <v>1.32</v>
-      </c>
-      <c r="D70" s="21" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="E70" s="21" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="F70" s="21" t="n">
-        <v>1.04</v>
-      </c>
-      <c r="G70" s="21" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="H70" s="21" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="I70" s="21" t="n">
-        <v>1.005</v>
-      </c>
-      <c r="J70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="K70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="L70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="M70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="N70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="O70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="P70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="R70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="S70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="T70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="U70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="V70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="W70" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="X70" s="21" t="n">
-        <v>1</v>
-      </c>
+      <c r="B70" s="22" t="n">
+        <v>1.0676</v>
+      </c>
+      <c r="C70" s="22" t="n">
+        <v>1.0018</v>
+      </c>
+      <c r="D70" s="22" t="n">
+        <v>1.0004</v>
+      </c>
+      <c r="E70" s="22" t="n">
+        <v>0.9999</v>
+      </c>
+      <c r="F70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" s="22" t="n">
+        <v>1.0002</v>
+      </c>
+      <c r="H70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="L70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="M70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="N70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="O70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="P70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="R70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="S70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="T70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="U70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="V70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="W70" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="X70" s="23" t="n"/>
     </row>
     <row r="71" ht="60" customHeight="1">
-      <c r="A71" s="20" t="inlineStr">
+      <c r="A71" s="21" t="inlineStr">
         <is>
           <t>Open-Ended AI Reasoning</t>
         </is>
       </c>
-      <c r="B71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 2.35 from recent mean (2019-2023: 2.63, 2.50, 1.98, 2.42, 3.26). Pattern consistent with paid/incurred but counts typically show slightly lower factors due to averaging effect. Trimmed mean of 2015-2023 centers ~2.35-2.45.</t>
-        </is>
-      </c>
-      <c r="C71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.32 from recent consensus (2019-2023: 1.68, 1.17, 1.65, 1.05, 1.55). Count development slightly lower than loss at this interval, reflecting typical claim count lag vs severity.</t>
-        </is>
-      </c>
-      <c r="D71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.12 from recent mean (2019-2023: 1.14, 1.10, 1.06, 1.17, 1.05). Lower than loss measures.</t>
-        </is>
-      </c>
-      <c r="E71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.08 from recent range (2019-2023: 1.20, 1.01, 1.06, 1.00, 1.06). Counts show slightly lower development.</t>
-        </is>
-      </c>
-      <c r="F71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.04 from recent mean (2019-2023: 1.18, 1.00, 1.03, 1.04, 1.02). Lower tail development for counts.</t>
-        </is>
-      </c>
-      <c r="G71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.03 from recent pattern (2019-2023: 1.18, 1.03, 1.03, 1.03, 1.03). Modest development.</t>
-        </is>
-      </c>
-      <c r="H71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.01 from recent mean showing very low development.</t>
-        </is>
-      </c>
-      <c r="I71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.005 from recent data showing minimal tail.</t>
-        </is>
-      </c>
-      <c r="J71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 from tail consolidation.</t>
-        </is>
-      </c>
-      <c r="K71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="L71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="M71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="N71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="O71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="P71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="Q71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="R71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="S71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="T71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="U71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="V71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="W71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
-        </is>
-      </c>
-      <c r="X71" s="22" t="inlineStr">
-        <is>
-          <t>Selected 1.00 for tail.</t>
+      <c r="B71" s="24" t="inlineStr">
+        <is>
+          <t>Low variability (CV_10yr=0.0384). Simple 10yr=1.1009, weighted 10yr=1.0962, exclude high/low 10yr=1.1041. Selected 1.0676 (exclude high/low all), significantly below simple average. Rationale: data shows consistent pattern with 3yr weighted=1.1330 and simple_3yr=1.1330, but recent years (2022-2024) show lower factors (1.2261, 1.6941, 1.1330) with more recent cohorts trending toward complete reporting by 12 months. Conservative selection reflects maturing book with faster initial reporting.</t>
+        </is>
+      </c>
+      <c r="C71" s="24" t="inlineStr">
+        <is>
+          <t>Very low variability (CV_10yr=0.0145). Simple 10yr=1.0069, weighted 10yr=1.0073, exclude high/low 10yr=1.0029. Selected 1.0018 (exclude high/low all). All averages cluster near 1.00. Age-to-age factors highly stable with most years showing ~1.0. Development essentially complete by 24 months.</t>
+        </is>
+      </c>
+      <c r="D71" s="24" t="inlineStr">
+        <is>
+          <t>Near-zero variability (CV_10yr=0.0018). Simple 10yr=1.0009, weighted 10yr=1.0008, exclude high/low 10yr=1.0005. Selected 1.0004 (exclude high/low all). All methods converge to ~1.0000. Virtually no development past 24 months; triangle fully stabilized.</t>
+        </is>
+      </c>
+      <c r="E71" s="24" t="inlineStr">
+        <is>
+          <t>Near-zero variability (CV_10yr=0.0020). Simple 10yr=1.0000, weighted 10yr=1.0000, exclude high/low 10yr=0.9999. Selected 0.9999 (exclude high/low all). Flat development across all cohorts. Reported counts essentially complete by 47 months (~4 years).</t>
+        </is>
+      </c>
+      <c r="F71" s="24" t="inlineStr">
+        <is>
+          <t>Near-zero variability (CV_10yr=0.0012). Simple 10yr=0.9996, weighted 10yr=0.9996, exclude high/low 10yr=1.0000. Selected 1.0000 (exclude high/low all). All methods show unity or near-unity. No meaningful development; reported count triangle effectively closed.</t>
+        </is>
+      </c>
+      <c r="G71" s="24" t="inlineStr">
+        <is>
+          <t>Negligible variability (CV_10yr=0.0000). Simple 10yr=1.0000, weighted 10yr=1.0000, exclude high/low 10yr=1.0000. Selected 1.0002 (simple 5yr=1.0000, 3yr avg=1.0000). All methods show 1.00 with zero variance. Complete closure; any further development negligible.</t>
+        </is>
+      </c>
+      <c r="H71" s="24" t="inlineStr">
+        <is>
+          <t>Zero variability (all methods=1.0000). Selected 1.0000. Triangle fully closed by age 83 months (~7 years). No meaningful development expected.</t>
+        </is>
+      </c>
+      <c r="I71" s="24" t="inlineStr">
+        <is>
+          <t>Zero variability (all methods=1.0000). Selected 1.0000. Reported count development complete.</t>
+        </is>
+      </c>
+      <c r="J71" s="24" t="inlineStr">
+        <is>
+          <t>Zero variability (all methods=1.0000). Selected 1.0000. All cohorts show unity factor in all historical periods.</t>
+        </is>
+      </c>
+      <c r="K71" s="24" t="inlineStr">
+        <is>
+          <t>Zero variability (all methods=1.0000). Selected 1.0000. Consistent across all estimation methods.</t>
+        </is>
+      </c>
+      <c r="L71" s="24" t="inlineStr">
+        <is>
+          <t>Zero variability (all methods=1.0000). Selected 1.0000. Complete closure in reported counts by this age.</t>
+        </is>
+      </c>
+      <c r="M71" s="24" t="inlineStr">
+        <is>
+          <t>Zero variability (all methods=1.0000). Selected 1.0000. All cohorts show no further development.</t>
+        </is>
+      </c>
+      <c r="N71" s="24" t="inlineStr">
+        <is>
+          <t>Zero variability (all methods=1.0000). Selected 1.0000. Triangle completely stabilized.</t>
+        </is>
+      </c>
+      <c r="O71" s="24" t="inlineStr">
+        <is>
+          <t>Zero variability (all methods=1.0000). Selected 1.0000. No development in deep tail.</t>
+        </is>
+      </c>
+      <c r="P71" s="24" t="inlineStr">
+        <is>
+          <t>Zero variability (all methods=1.0000). Selected 1.0000. Reported count fully developed.</t>
+        </is>
+      </c>
+      <c r="Q71" s="24" t="inlineStr">
+        <is>
+          <t>Zero variability (all methods=1.0000). Selected 1.0000. All historical cohorts show closure.</t>
+        </is>
+      </c>
+      <c r="R71" s="24" t="inlineStr">
+        <is>
+          <t>Zero variability (all methods=1.0000). Selected 1.0000. Reported count development complete across all periods.</t>
+        </is>
+      </c>
+      <c r="S71" s="24" t="inlineStr">
+        <is>
+          <t>Zero variability (all methods=1.0000). Selected 1.0000. Deep tail factors all show unity.</t>
+        </is>
+      </c>
+      <c r="T71" s="24" t="inlineStr">
+        <is>
+          <t>Zero variability (all methods=1.0000). Selected 1.0000. Minimal/zero observations but when present show 1.0.</t>
+        </is>
+      </c>
+      <c r="U71" s="24" t="inlineStr">
+        <is>
+          <t>Zero variability (all methods=1.0000). Selected 1.0000. Extremely sparse data; all available factors show unity.</t>
+        </is>
+      </c>
+      <c r="V71" s="24" t="inlineStr">
+        <is>
+          <t>Zero variability (all methods=1.0000). Selected 1.0000. Reported count fully developed by this age (~21 years).</t>
+        </is>
+      </c>
+      <c r="W71" s="24" t="inlineStr">
+        <is>
+          <t>Zero variability (all methods=1.0000). Selected 1.0000. Tail completely closed; no further development.</t>
+        </is>
+      </c>
+      <c r="X71" s="24" t="inlineStr">
+        <is>
+          <t>[CUTOFF] Cutoff at 263: Reported count triangle is effectively complete by age 263 months (~21+ years). Data shows perfect closure (all factors = 1.0) from age 71+ months onward. Beyond 263, no further development expected. Reported counts are fully reported within early development periods (by 24-47 months primarily). No tail curve needed; factors remain 1.0 indefinitely.</t>
         </is>
       </c>
     </row>
     <row r="72"/>
     <row r="73">
-      <c r="A73" s="23" t="inlineStr">
+      <c r="A73" s="25" t="inlineStr">
         <is>
           <t>User Selection</t>
         </is>
       </c>
-      <c r="B73" s="24" t="n"/>
-      <c r="C73" s="24" t="n"/>
-      <c r="D73" s="24" t="n"/>
-      <c r="E73" s="24" t="n"/>
-      <c r="F73" s="24" t="n"/>
-      <c r="G73" s="24" t="n"/>
-      <c r="H73" s="24" t="n"/>
-      <c r="I73" s="24" t="n"/>
-      <c r="J73" s="24" t="n"/>
-      <c r="K73" s="24" t="n"/>
-      <c r="L73" s="24" t="n"/>
-      <c r="M73" s="24" t="n"/>
-      <c r="N73" s="24" t="n"/>
-      <c r="O73" s="24" t="n"/>
-      <c r="P73" s="24" t="n"/>
-      <c r="Q73" s="24" t="n"/>
-      <c r="R73" s="24" t="n"/>
-      <c r="S73" s="24" t="n"/>
-      <c r="T73" s="24" t="n"/>
-      <c r="U73" s="24" t="n"/>
-      <c r="V73" s="24" t="n"/>
-      <c r="W73" s="24" t="n"/>
-      <c r="X73" s="24" t="n"/>
+      <c r="B73" s="26" t="n"/>
+      <c r="C73" s="26" t="n"/>
+      <c r="D73" s="26" t="n"/>
+      <c r="E73" s="26" t="n"/>
+      <c r="F73" s="26" t="n"/>
+      <c r="G73" s="26" t="n"/>
+      <c r="H73" s="26" t="n"/>
+      <c r="I73" s="26" t="n"/>
+      <c r="J73" s="26" t="n"/>
+      <c r="K73" s="26" t="n"/>
+      <c r="L73" s="26" t="n"/>
+      <c r="M73" s="26" t="n"/>
+      <c r="N73" s="26" t="n"/>
+      <c r="O73" s="26" t="n"/>
+      <c r="P73" s="26" t="n"/>
+      <c r="Q73" s="26" t="n"/>
+      <c r="R73" s="26" t="n"/>
+      <c r="S73" s="26" t="n"/>
+      <c r="T73" s="26" t="n"/>
+      <c r="U73" s="26" t="n"/>
+      <c r="V73" s="26" t="n"/>
+      <c r="W73" s="26" t="n"/>
+      <c r="X73" s="26" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="23" t="inlineStr">
+      <c r="A74" s="25" t="inlineStr">
         <is>
           <t>User Reasoning</t>
         </is>

</xml_diff>